<commit_message>
implemented gas phase transport
</commit_message>
<xml_diff>
--- a/southern_europe/italy_data/network_capex_metrics/capex_defined_per_arc_large.xlsx
+++ b/southern_europe/italy_data/network_capex_metrics/capex_defined_per_arc_large.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gamma1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gamma2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gamma3" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gamma4" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="gamma1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="gamma2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="gamma3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="gamma4" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,150 +420,150 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="n">
+      <c r="B1" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="n">
+      <c r="C1" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="n">
+      <c r="D1" t="n">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="n">
+      <c r="E1" t="n">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="n">
+      <c r="F1" t="n">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="n">
+      <c r="G1" t="n">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="n">
+      <c r="H1" t="n">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="n">
+      <c r="I1" t="n">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="n">
+      <c r="J1" t="n">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="n">
+      <c r="K1" t="n">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="n">
+      <c r="L1" t="n">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="n">
+      <c r="M1" t="n">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="n">
+      <c r="N1" t="n">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="n">
+      <c r="O1" t="n">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="n">
+      <c r="P1" t="n">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="n">
+      <c r="Q1" t="n">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="n">
+      <c r="R1" t="n">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="n">
+      <c r="S1" t="n">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="n">
+      <c r="T1" t="n">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="n">
+      <c r="U1" t="n">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="n">
+      <c r="V1" t="n">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="n">
+      <c r="W1" t="n">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="n">
+      <c r="X1" t="n">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="n">
+      <c r="Y1" t="n">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="n">
+      <c r="Z1" t="n">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="n">
+      <c r="AA1" t="n">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="n">
+      <c r="AB1" t="n">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="n">
+      <c r="AC1" t="n">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="n">
+      <c r="AD1" t="n">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="n">
+      <c r="AE1" t="n">
         <v>30</v>
       </c>
-      <c r="AF1" s="1" t="n">
+      <c r="AF1" t="n">
         <v>31</v>
       </c>
-      <c r="AG1" s="1" t="n">
+      <c r="AG1" t="n">
         <v>32</v>
       </c>
-      <c r="AH1" s="1" t="n">
+      <c r="AH1" t="n">
         <v>33</v>
       </c>
-      <c r="AI1" s="1" t="n">
+      <c r="AI1" t="n">
         <v>34</v>
       </c>
-      <c r="AJ1" s="1" t="n">
+      <c r="AJ1" t="n">
         <v>35</v>
       </c>
-      <c r="AK1" s="1" t="n">
+      <c r="AK1" t="n">
         <v>36</v>
       </c>
-      <c r="AL1" s="1" t="n">
+      <c r="AL1" t="n">
         <v>37</v>
       </c>
-      <c r="AM1" s="1" t="n">
+      <c r="AM1" t="n">
         <v>38</v>
       </c>
-      <c r="AN1" s="1" t="n">
+      <c r="AN1" t="n">
         <v>39</v>
       </c>
-      <c r="AO1" s="1" t="n">
+      <c r="AO1" t="n">
         <v>40</v>
       </c>
-      <c r="AP1" s="1" t="n">
+      <c r="AP1" t="n">
         <v>41</v>
       </c>
-      <c r="AQ1" s="1" t="n">
+      <c r="AQ1" t="n">
         <v>42</v>
       </c>
-      <c r="AR1" s="1" t="n">
+      <c r="AR1" t="n">
         <v>43</v>
       </c>
-      <c r="AS1" s="1" t="n">
+      <c r="AS1" t="n">
         <v>44</v>
       </c>
-      <c r="AT1" s="1" t="n">
+      <c r="AT1" t="n">
         <v>45</v>
       </c>
-      <c r="AU1" s="1" t="n">
+      <c r="AU1" t="n">
         <v>46</v>
       </c>
-      <c r="AV1" s="1" t="n">
+      <c r="AV1" t="n">
         <v>47</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="n">
@@ -585,7 +573,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>47146678.639</v>
+        <v>78719857.325</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -721,7 +709,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
       <c r="B3" t="n">
@@ -752,7 +740,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>102897360.093</v>
+        <v>166946295.967</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -863,11 +851,11 @@
         <v>0</v>
       </c>
       <c r="AV3" t="n">
-        <v>12368660.665</v>
+        <v>13671245.914</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
       <c r="B4" t="n">
@@ -889,13 +877,13 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>30274934.652</v>
+        <v>51383912.857</v>
       </c>
       <c r="I4" t="n">
-        <v>25734215.382</v>
+        <v>42501259.047</v>
       </c>
       <c r="J4" t="n">
-        <v>30570505.833</v>
+        <v>52867280.881</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -1013,7 +1001,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
       <c r="B5" t="n">
@@ -1029,7 +1017,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>14181812.724</v>
+        <v>12618154.122</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -1047,10 +1035,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>36253967.123</v>
+        <v>46825310.452</v>
       </c>
       <c r="M5" t="n">
-        <v>40906488.824</v>
+        <v>67285230.771</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -1159,7 +1147,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
       <c r="B6" t="n">
@@ -1178,7 +1166,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>23376882.44</v>
+        <v>29649765.414</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -1193,10 +1181,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>29957645.119</v>
+        <v>39173678.268</v>
       </c>
       <c r="M6" t="n">
-        <v>35150745.711</v>
+        <v>54920778.79</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -1305,7 +1293,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
       <c r="B7" t="n">
@@ -1327,7 +1315,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>14677753.771</v>
+        <v>15049863.318</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -1342,10 +1330,10 @@
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>27054490.74</v>
+        <v>33359701.108</v>
       </c>
       <c r="N7" t="n">
-        <v>21791693.253</v>
+        <v>22770316.028</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
@@ -1451,7 +1439,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>7</v>
       </c>
       <c r="B8" t="n">
@@ -1470,13 +1458,13 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>12102777.914</v>
+        <v>13161208.215</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>16137717.497</v>
+        <v>17056305.51</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -1491,16 +1479,16 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>23033001.505</v>
+        <v>25751956.704</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>31059093.027</v>
+        <v>48319635.114</v>
       </c>
       <c r="Q8" t="n">
-        <v>34882368.619</v>
+        <v>58533852.159</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1597,7 +1585,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>8</v>
       </c>
       <c r="B9" t="n">
@@ -1619,13 +1607,13 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>14308629.824</v>
+        <v>15525931.091</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>18510403.418</v>
+        <v>21682694.404</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -1637,16 +1625,16 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>25911693.289</v>
+        <v>36729186.476</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>35029214.04</v>
+        <v>53376399.13</v>
       </c>
       <c r="Q9" t="n">
-        <v>31751132.502</v>
+        <v>51016697.784</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
@@ -1743,7 +1731,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>9</v>
       </c>
       <c r="B10" t="n">
@@ -1768,13 +1756,13 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>16887485.282</v>
+        <v>20043014.289</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>45405895.414</v>
+        <v>76167400.94499999</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -1789,10 +1777,10 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>34164666.446</v>
+        <v>60397802.079</v>
       </c>
       <c r="Q10" t="n">
-        <v>25322132.215</v>
+        <v>42273418.771</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
@@ -1804,10 +1792,10 @@
         <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>49351702.381</v>
+        <v>76976861.234</v>
       </c>
       <c r="V10" t="n">
-        <v>61853766.218</v>
+        <v>104816477.374</v>
       </c>
       <c r="W10" t="n">
         <v>0</v>
@@ -1889,7 +1877,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>10</v>
       </c>
       <c r="B11" t="n">
@@ -1917,7 +1905,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>32632639.075</v>
+        <v>58272409.302</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -1953,7 +1941,7 @@
         <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>69494855.698</v>
+        <v>96462615.14</v>
       </c>
       <c r="W11" t="n">
         <v>0</v>
@@ -2035,7 +2023,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" t="n">
         <v>11</v>
       </c>
       <c r="B12" t="n">
@@ -2072,7 +2060,7 @@
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>28774492.734</v>
+        <v>28089579.407</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -2087,10 +2075,10 @@
         <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>28744769.78</v>
+        <v>30182953.108</v>
       </c>
       <c r="S12" t="n">
-        <v>33891249.152</v>
+        <v>45907376.545</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -2181,7 +2169,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" t="n">
         <v>12</v>
       </c>
       <c r="B13" t="n">
@@ -2200,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>17685041.419</v>
+        <v>24408713.242</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -2224,7 +2212,7 @@
         <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>19238875.127</v>
+        <v>13844532.627</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
@@ -2236,7 +2224,7 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>30751100.547</v>
+        <v>31526047.884</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -2327,7 +2315,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="n">
         <v>13</v>
       </c>
       <c r="B14" t="n">
@@ -2349,7 +2337,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>17932449.736</v>
+        <v>21274243.959</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -2370,10 +2358,10 @@
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>21928247.775</v>
+        <v>19114878.449</v>
       </c>
       <c r="P14" t="n">
-        <v>23334145.294</v>
+        <v>21317775.079</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
@@ -2473,7 +2461,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" t="n">
         <v>14</v>
       </c>
       <c r="B15" t="n">
@@ -2513,13 +2501,13 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>11680468.929</v>
+        <v>12598202.967</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>19462634.449</v>
+        <v>10768201.645</v>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
@@ -2531,7 +2519,7 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>33363977.414</v>
+        <v>42837537.263</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -2543,7 +2531,7 @@
         <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>58607423.206</v>
+        <v>85298545.04899999</v>
       </c>
       <c r="Y15" t="n">
         <v>0</v>
@@ -2619,7 +2607,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" t="n">
         <v>15</v>
       </c>
       <c r="B16" t="n">
@@ -2668,7 +2656,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>29029981.388</v>
+        <v>39638437.645</v>
       </c>
       <c r="R16" t="n">
         <v>0</v>
@@ -2680,7 +2668,7 @@
         <v>0</v>
       </c>
       <c r="U16" t="n">
-        <v>38702083.624</v>
+        <v>67279421.88</v>
       </c>
       <c r="V16" t="n">
         <v>0</v>
@@ -2689,7 +2677,7 @@
         <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>46530999.851</v>
+        <v>69023910.601</v>
       </c>
       <c r="Y16" t="n">
         <v>0</v>
@@ -2765,7 +2753,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" t="n">
         <v>16</v>
       </c>
       <c r="B17" t="n">
@@ -2826,7 +2814,7 @@
         <v>0</v>
       </c>
       <c r="U17" t="n">
-        <v>24619499.785</v>
+        <v>34698471.289</v>
       </c>
       <c r="V17" t="n">
         <v>0</v>
@@ -2911,7 +2899,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" t="n">
         <v>17</v>
       </c>
       <c r="B18" t="n">
@@ -2966,7 +2954,7 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>25473648.057</v>
+        <v>24763255.977</v>
       </c>
       <c r="T18" t="n">
         <v>0</v>
@@ -3047,7 +3035,7 @@
         <v>0</v>
       </c>
       <c r="AT18" t="n">
-        <v>27250547.431</v>
+        <v>27659449.998</v>
       </c>
       <c r="AU18" t="n">
         <v>0</v>
@@ -3057,7 +3045,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" t="n">
         <v>18</v>
       </c>
       <c r="B19" t="n">
@@ -3094,13 +3082,13 @@
         <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>17564113.238</v>
+        <v>20605786.177</v>
       </c>
       <c r="N19" t="n">
         <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>29748132.282</v>
+        <v>31731479.262</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
@@ -3115,7 +3103,7 @@
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>18868594.966</v>
+        <v>15088951.669</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
@@ -3193,7 +3181,7 @@
         <v>0</v>
       </c>
       <c r="AT19" t="n">
-        <v>22854163.383</v>
+        <v>20932711.3</v>
       </c>
       <c r="AU19" t="n">
         <v>0</v>
@@ -3203,7 +3191,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" t="n">
         <v>19</v>
       </c>
       <c r="B20" t="n">
@@ -3246,7 +3234,7 @@
         <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>21467210.927</v>
+        <v>30412140.677</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
@@ -3258,22 +3246,22 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>10758138.638</v>
+        <v>10572888.913</v>
       </c>
       <c r="T20" t="n">
         <v>0</v>
       </c>
       <c r="U20" t="n">
-        <v>43243196.048</v>
+        <v>73496610.985</v>
       </c>
       <c r="V20" t="n">
         <v>0</v>
       </c>
       <c r="W20" t="n">
-        <v>38259931.007</v>
+        <v>48809510.429</v>
       </c>
       <c r="X20" t="n">
-        <v>36208657.378</v>
+        <v>60032899.146</v>
       </c>
       <c r="Y20" t="n">
         <v>0</v>
@@ -3349,7 +3337,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" t="n">
         <v>20</v>
       </c>
       <c r="B21" t="n">
@@ -3419,16 +3407,16 @@
         <v>0</v>
       </c>
       <c r="X21" t="n">
-        <v>41704820.458</v>
+        <v>71112868.38</v>
       </c>
       <c r="Y21" t="n">
         <v>0</v>
       </c>
       <c r="Z21" t="n">
-        <v>34973089.916</v>
+        <v>61101544.146</v>
       </c>
       <c r="AA21" t="n">
-        <v>75842152.90099999</v>
+        <v>125330168.992</v>
       </c>
       <c r="AB21" t="n">
         <v>0</v>
@@ -3482,7 +3470,7 @@
         <v>0</v>
       </c>
       <c r="AS21" t="n">
-        <v>51074158.37</v>
+        <v>75371178.65700001</v>
       </c>
       <c r="AT21" t="n">
         <v>0</v>
@@ -3495,7 +3483,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" t="n">
         <v>21</v>
       </c>
       <c r="B22" t="n">
@@ -3556,7 +3544,7 @@
         <v>0</v>
       </c>
       <c r="U22" t="n">
-        <v>23247683.287</v>
+        <v>25539984.938</v>
       </c>
       <c r="V22" t="n">
         <v>0</v>
@@ -3571,7 +3559,7 @@
         <v>0</v>
       </c>
       <c r="Z22" t="n">
-        <v>34584825.496</v>
+        <v>54052199.155</v>
       </c>
       <c r="AA22" t="n">
         <v>0</v>
@@ -3641,7 +3629,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" t="n">
         <v>22</v>
       </c>
       <c r="B23" t="n">
@@ -3699,10 +3687,10 @@
         <v>0</v>
       </c>
       <c r="T23" t="n">
-        <v>24590932.875</v>
+        <v>34063895.868</v>
       </c>
       <c r="U23" t="n">
-        <v>57057466.637</v>
+        <v>84500283.248</v>
       </c>
       <c r="V23" t="n">
         <v>0</v>
@@ -3711,7 +3699,7 @@
         <v>0</v>
       </c>
       <c r="X23" t="n">
-        <v>27206367.911</v>
+        <v>31957728.567</v>
       </c>
       <c r="Y23" t="n">
         <v>0</v>
@@ -3787,7 +3775,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" t="n">
         <v>23</v>
       </c>
       <c r="B24" t="n">
@@ -3848,7 +3836,7 @@
         <v>0</v>
       </c>
       <c r="U24" t="n">
-        <v>36827207.323</v>
+        <v>63729848.081</v>
       </c>
       <c r="V24" t="n">
         <v>0</v>
@@ -3860,7 +3848,7 @@
         <v>0</v>
       </c>
       <c r="Y24" t="n">
-        <v>15985965.45</v>
+        <v>12452131.841</v>
       </c>
       <c r="Z24" t="n">
         <v>0</v>
@@ -3926,14 +3914,14 @@
         <v>0</v>
       </c>
       <c r="AU24" t="n">
-        <v>16313596.568</v>
+        <v>13122040.814</v>
       </c>
       <c r="AV24" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" t="n">
         <v>24</v>
       </c>
       <c r="B25" t="n">
@@ -4003,7 +3991,7 @@
         <v>0</v>
       </c>
       <c r="X25" t="n">
-        <v>9421460.120999999</v>
+        <v>9064089.668</v>
       </c>
       <c r="Y25" t="n">
         <v>0</v>
@@ -4012,7 +4000,7 @@
         <v>0</v>
       </c>
       <c r="AA25" t="n">
-        <v>41655280.905</v>
+        <v>70727198.957</v>
       </c>
       <c r="AB25" t="n">
         <v>0</v>
@@ -4072,14 +4060,14 @@
         <v>0</v>
       </c>
       <c r="AU25" t="n">
-        <v>17366215.261</v>
+        <v>9665014.898</v>
       </c>
       <c r="AV25" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" t="n">
         <v>25</v>
       </c>
       <c r="B26" t="n">
@@ -4161,13 +4149,13 @@
         <v>0</v>
       </c>
       <c r="AB26" t="n">
-        <v>31731212.707</v>
+        <v>55240886.296</v>
       </c>
       <c r="AC26" t="n">
         <v>0</v>
       </c>
       <c r="AD26" t="n">
-        <v>57146245.037</v>
+        <v>102365063.311</v>
       </c>
       <c r="AE26" t="n">
         <v>0</v>
@@ -4212,7 +4200,7 @@
         <v>0</v>
       </c>
       <c r="AS26" t="n">
-        <v>20367253.893</v>
+        <v>24128912.349</v>
       </c>
       <c r="AT26" t="n">
         <v>0</v>
@@ -4225,7 +4213,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" t="n">
         <v>26</v>
       </c>
       <c r="B27" t="n">
@@ -4307,19 +4295,19 @@
         <v>0</v>
       </c>
       <c r="AB27" t="n">
-        <v>50651241.221</v>
+        <v>88723408.71799999</v>
       </c>
       <c r="AC27" t="n">
         <v>0</v>
       </c>
       <c r="AD27" t="n">
-        <v>49463717.279</v>
+        <v>73379041.83</v>
       </c>
       <c r="AE27" t="n">
-        <v>69486393.743</v>
+        <v>114162995.818</v>
       </c>
       <c r="AF27" t="n">
-        <v>38277302.28</v>
+        <v>66786176.666</v>
       </c>
       <c r="AG27" t="n">
         <v>0</v>
@@ -4328,7 +4316,7 @@
         <v>0</v>
       </c>
       <c r="AI27" t="n">
-        <v>50879396.057</v>
+        <v>79428010.83400001</v>
       </c>
       <c r="AJ27" t="n">
         <v>0</v>
@@ -4358,7 +4346,7 @@
         <v>0</v>
       </c>
       <c r="AS27" t="n">
-        <v>37632393.684</v>
+        <v>65901211.034</v>
       </c>
       <c r="AT27" t="n">
         <v>0</v>
@@ -4371,7 +4359,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" t="n">
         <v>27</v>
       </c>
       <c r="B28" t="n">
@@ -4450,7 +4438,7 @@
         <v>0</v>
       </c>
       <c r="AA28" t="n">
-        <v>45945354.108</v>
+        <v>81131094.20200001</v>
       </c>
       <c r="AB28" t="n">
         <v>0</v>
@@ -4459,10 +4447,10 @@
         <v>0</v>
       </c>
       <c r="AD28" t="n">
-        <v>33781763.026</v>
+        <v>56892764.744</v>
       </c>
       <c r="AE28" t="n">
-        <v>32290810.919</v>
+        <v>49754918.165</v>
       </c>
       <c r="AF28" t="n">
         <v>0</v>
@@ -4517,7 +4505,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" t="n">
         <v>28</v>
       </c>
       <c r="B29" t="n">
@@ -4596,7 +4584,7 @@
         <v>0</v>
       </c>
       <c r="AA29" t="n">
-        <v>96496155.44599999</v>
+        <v>169150365.72</v>
       </c>
       <c r="AB29" t="n">
         <v>0</v>
@@ -4614,13 +4602,13 @@
         <v>0</v>
       </c>
       <c r="AG29" t="n">
-        <v>91942218.567</v>
+        <v>148210174.515</v>
       </c>
       <c r="AH29" t="n">
-        <v>68740572.347</v>
+        <v>115226114.605</v>
       </c>
       <c r="AI29" t="n">
-        <v>95619421.421</v>
+        <v>169981376.333</v>
       </c>
       <c r="AJ29" t="n">
         <v>0</v>
@@ -4663,7 +4651,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" t="n">
         <v>29</v>
       </c>
       <c r="B30" t="n">
@@ -4754,7 +4742,7 @@
         <v>0</v>
       </c>
       <c r="AE30" t="n">
-        <v>25885289.455</v>
+        <v>42967185.69</v>
       </c>
       <c r="AF30" t="n">
         <v>0</v>
@@ -4769,13 +4757,13 @@
         <v>0</v>
       </c>
       <c r="AJ30" t="n">
-        <v>50737752.276</v>
+        <v>89603855.911</v>
       </c>
       <c r="AK30" t="n">
         <v>0</v>
       </c>
       <c r="AL30" t="n">
-        <v>48154728.177</v>
+        <v>72072622.265</v>
       </c>
       <c r="AM30" t="n">
         <v>0</v>
@@ -4809,7 +4797,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" t="n">
         <v>30</v>
       </c>
       <c r="B31" t="n">
@@ -4897,7 +4885,7 @@
         <v>0</v>
       </c>
       <c r="AD31" t="n">
-        <v>23233076.885</v>
+        <v>39220154.935</v>
       </c>
       <c r="AE31" t="n">
         <v>0</v>
@@ -4915,13 +4903,13 @@
         <v>0</v>
       </c>
       <c r="AJ31" t="n">
-        <v>41266624.505</v>
+        <v>69896552.086</v>
       </c>
       <c r="AK31" t="n">
         <v>0</v>
       </c>
       <c r="AL31" t="n">
-        <v>39248201.255</v>
+        <v>67007912.995</v>
       </c>
       <c r="AM31" t="n">
         <v>0</v>
@@ -4955,7 +4943,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" t="n">
         <v>31</v>
       </c>
       <c r="B32" t="n">
@@ -5058,7 +5046,7 @@
         <v>0</v>
       </c>
       <c r="AI32" t="n">
-        <v>22397745.017</v>
+        <v>24837139.994</v>
       </c>
       <c r="AJ32" t="n">
         <v>0</v>
@@ -5067,7 +5055,7 @@
         <v>0</v>
       </c>
       <c r="AL32" t="n">
-        <v>66471062.077</v>
+        <v>109174389.664</v>
       </c>
       <c r="AM32" t="n">
         <v>0</v>
@@ -5101,7 +5089,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" t="n">
         <v>32</v>
       </c>
       <c r="B33" t="n">
@@ -5180,7 +5168,7 @@
         <v>0</v>
       </c>
       <c r="AA33" t="n">
-        <v>24760989.774</v>
+        <v>29858452.336</v>
       </c>
       <c r="AB33" t="n">
         <v>0</v>
@@ -5247,7 +5235,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" t="n">
         <v>33</v>
       </c>
       <c r="B34" t="n">
@@ -5350,19 +5338,19 @@
         <v>0</v>
       </c>
       <c r="AI34" t="n">
-        <v>36078389.239</v>
+        <v>63342430.989</v>
       </c>
       <c r="AJ34" t="n">
         <v>0</v>
       </c>
       <c r="AK34" t="n">
-        <v>23063409.44</v>
+        <v>27755149.855</v>
       </c>
       <c r="AL34" t="n">
         <v>0</v>
       </c>
       <c r="AM34" t="n">
-        <v>28905497.591</v>
+        <v>51024875.892</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -5393,7 +5381,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" t="n">
         <v>34</v>
       </c>
       <c r="B35" t="n">
@@ -5487,7 +5475,7 @@
         <v>0</v>
       </c>
       <c r="AF35" t="n">
-        <v>16948730.146</v>
+        <v>20157316.823</v>
       </c>
       <c r="AG35" t="n">
         <v>0</v>
@@ -5508,7 +5496,7 @@
         <v>0</v>
       </c>
       <c r="AM35" t="n">
-        <v>17298625.641</v>
+        <v>23131272.452</v>
       </c>
       <c r="AN35" t="n">
         <v>0</v>
@@ -5539,7 +5527,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" t="n">
         <v>35</v>
       </c>
       <c r="B36" t="n">
@@ -5651,7 +5639,7 @@
         <v>0</v>
       </c>
       <c r="AL36" t="n">
-        <v>17829092.333</v>
+        <v>20453703.872</v>
       </c>
       <c r="AM36" t="n">
         <v>0</v>
@@ -5685,7 +5673,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" t="n">
         <v>36</v>
       </c>
       <c r="B37" t="n">
@@ -5785,10 +5773,10 @@
         <v>0</v>
       </c>
       <c r="AH37" t="n">
-        <v>17521764.04</v>
+        <v>22682238.651</v>
       </c>
       <c r="AI37" t="n">
-        <v>34401862.527</v>
+        <v>61150272.942</v>
       </c>
       <c r="AJ37" t="n">
         <v>0</v>
@@ -5800,7 +5788,7 @@
         <v>0</v>
       </c>
       <c r="AM37" t="n">
-        <v>24411936.601</v>
+        <v>39439397.523</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -5831,7 +5819,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" t="n">
         <v>37</v>
       </c>
       <c r="B38" t="n">
@@ -5958,7 +5946,7 @@
         <v>0</v>
       </c>
       <c r="AQ38" t="n">
-        <v>16662663.606</v>
+        <v>17722478.754</v>
       </c>
       <c r="AR38" t="n">
         <v>0</v>
@@ -5977,7 +5965,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" t="n">
         <v>38</v>
       </c>
       <c r="B39" t="n">
@@ -6080,7 +6068,7 @@
         <v>0</v>
       </c>
       <c r="AI39" t="n">
-        <v>17298625.641</v>
+        <v>23131272.452</v>
       </c>
       <c r="AJ39" t="n">
         <v>0</v>
@@ -6123,7 +6111,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" t="n">
         <v>39</v>
       </c>
       <c r="B40" t="n">
@@ -6232,13 +6220,13 @@
         <v>0</v>
       </c>
       <c r="AK40" t="n">
-        <v>43672697.261</v>
+        <v>69901045.027</v>
       </c>
       <c r="AL40" t="n">
         <v>0</v>
       </c>
       <c r="AM40" t="n">
-        <v>49749046.706</v>
+        <v>88487003.76000001</v>
       </c>
       <c r="AN40" t="n">
         <v>0</v>
@@ -6269,7 +6257,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" t="n">
         <v>40</v>
       </c>
       <c r="B41" t="n">
@@ -6381,7 +6369,7 @@
         <v>0</v>
       </c>
       <c r="AL41" t="n">
-        <v>39170538.809</v>
+        <v>67782348.774</v>
       </c>
       <c r="AM41" t="n">
         <v>0</v>
@@ -6415,7 +6403,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" t="n">
         <v>41</v>
       </c>
       <c r="B42" t="n">
@@ -6524,13 +6512,13 @@
         <v>0</v>
       </c>
       <c r="AK42" t="n">
-        <v>77981115.33400001</v>
+        <v>142219609.658</v>
       </c>
       <c r="AL42" t="n">
         <v>0</v>
       </c>
       <c r="AM42" t="n">
-        <v>78666062.994</v>
+        <v>140736821.285</v>
       </c>
       <c r="AN42" t="n">
         <v>0</v>
@@ -6561,7 +6549,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" t="n">
         <v>42</v>
       </c>
       <c r="B43" t="n">
@@ -6707,7 +6695,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" t="n">
         <v>43</v>
       </c>
       <c r="B44" t="n">
@@ -6853,7 +6841,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" t="n">
         <v>44</v>
       </c>
       <c r="B45" t="n">
@@ -6929,19 +6917,19 @@
         <v>0</v>
       </c>
       <c r="Z45" t="n">
-        <v>18174964.191</v>
+        <v>21942902.07</v>
       </c>
       <c r="AA45" t="n">
         <v>0</v>
       </c>
       <c r="AB45" t="n">
-        <v>27086900.852</v>
+        <v>43088860.497</v>
       </c>
       <c r="AC45" t="n">
         <v>0</v>
       </c>
       <c r="AD45" t="n">
-        <v>50042925.935</v>
+        <v>74014768.458</v>
       </c>
       <c r="AE45" t="n">
         <v>0</v>
@@ -6999,7 +6987,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" t="n">
         <v>45</v>
       </c>
       <c r="B46" t="n">
@@ -7054,10 +7042,10 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>13732889.927</v>
+        <v>14743727.345</v>
       </c>
       <c r="T46" t="n">
-        <v>14646500.475</v>
+        <v>15956529.138</v>
       </c>
       <c r="U46" t="n">
         <v>0</v>
@@ -7066,10 +7054,10 @@
         <v>0</v>
       </c>
       <c r="W46" t="n">
-        <v>24749693.804</v>
+        <v>32727478.392</v>
       </c>
       <c r="X46" t="n">
-        <v>31295668.594</v>
+        <v>55196699.797</v>
       </c>
       <c r="Y46" t="n">
         <v>0</v>
@@ -7145,7 +7133,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" t="n">
         <v>46</v>
       </c>
       <c r="B47" t="n">
@@ -7218,13 +7206,13 @@
         <v>0</v>
       </c>
       <c r="Y47" t="n">
-        <v>9127851.335000001</v>
+        <v>6597618.651</v>
       </c>
       <c r="Z47" t="n">
-        <v>42133678.733</v>
+        <v>66911746.737</v>
       </c>
       <c r="AA47" t="n">
-        <v>40126720.576</v>
+        <v>68681860.649</v>
       </c>
       <c r="AB47" t="n">
         <v>0</v>
@@ -7278,7 +7266,7 @@
         <v>0</v>
       </c>
       <c r="AS47" t="n">
-        <v>39626175.353</v>
+        <v>67263117.831</v>
       </c>
       <c r="AT47" t="n">
         <v>0</v>
@@ -7291,14 +7279,14 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" t="n">
         <v>47</v>
       </c>
       <c r="B48" t="n">
         <v>0</v>
       </c>
       <c r="C48" t="n">
-        <v>21631321.332</v>
+        <v>19714851.841</v>
       </c>
       <c r="D48" t="n">
         <v>0</v>
@@ -7322,7 +7310,7 @@
         <v>0</v>
       </c>
       <c r="K48" t="n">
-        <v>90461257.274</v>
+        <v>159964881.304</v>
       </c>
       <c r="L48" t="n">
         <v>0</v>
@@ -7451,150 +7439,150 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="n">
+      <c r="B1" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="n">
+      <c r="C1" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="n">
+      <c r="D1" t="n">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="n">
+      <c r="E1" t="n">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="n">
+      <c r="F1" t="n">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="n">
+      <c r="G1" t="n">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="n">
+      <c r="H1" t="n">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="n">
+      <c r="I1" t="n">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="n">
+      <c r="J1" t="n">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="n">
+      <c r="K1" t="n">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="n">
+      <c r="L1" t="n">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="n">
+      <c r="M1" t="n">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="n">
+      <c r="N1" t="n">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="n">
+      <c r="O1" t="n">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="n">
+      <c r="P1" t="n">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="n">
+      <c r="Q1" t="n">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="n">
+      <c r="R1" t="n">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="n">
+      <c r="S1" t="n">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="n">
+      <c r="T1" t="n">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="n">
+      <c r="U1" t="n">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="n">
+      <c r="V1" t="n">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="n">
+      <c r="W1" t="n">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="n">
+      <c r="X1" t="n">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="n">
+      <c r="Y1" t="n">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="n">
+      <c r="Z1" t="n">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="n">
+      <c r="AA1" t="n">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="n">
+      <c r="AB1" t="n">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="n">
+      <c r="AC1" t="n">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="n">
+      <c r="AD1" t="n">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="n">
+      <c r="AE1" t="n">
         <v>30</v>
       </c>
-      <c r="AF1" s="1" t="n">
+      <c r="AF1" t="n">
         <v>31</v>
       </c>
-      <c r="AG1" s="1" t="n">
+      <c r="AG1" t="n">
         <v>32</v>
       </c>
-      <c r="AH1" s="1" t="n">
+      <c r="AH1" t="n">
         <v>33</v>
       </c>
-      <c r="AI1" s="1" t="n">
+      <c r="AI1" t="n">
         <v>34</v>
       </c>
-      <c r="AJ1" s="1" t="n">
+      <c r="AJ1" t="n">
         <v>35</v>
       </c>
-      <c r="AK1" s="1" t="n">
+      <c r="AK1" t="n">
         <v>36</v>
       </c>
-      <c r="AL1" s="1" t="n">
+      <c r="AL1" t="n">
         <v>37</v>
       </c>
-      <c r="AM1" s="1" t="n">
+      <c r="AM1" t="n">
         <v>38</v>
       </c>
-      <c r="AN1" s="1" t="n">
+      <c r="AN1" t="n">
         <v>39</v>
       </c>
-      <c r="AO1" s="1" t="n">
+      <c r="AO1" t="n">
         <v>40</v>
       </c>
-      <c r="AP1" s="1" t="n">
+      <c r="AP1" t="n">
         <v>41</v>
       </c>
-      <c r="AQ1" s="1" t="n">
+      <c r="AQ1" t="n">
         <v>42</v>
       </c>
-      <c r="AR1" s="1" t="n">
+      <c r="AR1" t="n">
         <v>43</v>
       </c>
-      <c r="AS1" s="1" t="n">
+      <c r="AS1" t="n">
         <v>44</v>
       </c>
-      <c r="AT1" s="1" t="n">
+      <c r="AT1" t="n">
         <v>45</v>
       </c>
-      <c r="AU1" s="1" t="n">
+      <c r="AU1" t="n">
         <v>46</v>
       </c>
-      <c r="AV1" s="1" t="n">
+      <c r="AV1" t="n">
         <v>47</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="n">
@@ -7604,7 +7592,7 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>87317.164</v>
+        <v>58306.519</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
@@ -7740,7 +7728,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
       <c r="B3" t="n">
@@ -7771,7 +7759,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>113154.366</v>
+        <v>118085.022</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -7882,11 +7870,11 @@
         <v>0</v>
       </c>
       <c r="AV3" t="n">
-        <v>57457.78</v>
+        <v>15128.797</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
       <c r="B4" t="n">
@@ -7908,13 +7896,13 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>76205.507</v>
+        <v>47343.345</v>
       </c>
       <c r="I4" t="n">
-        <v>72376.28599999999</v>
+        <v>39512.47</v>
       </c>
       <c r="J4" t="n">
-        <v>78235.64</v>
+        <v>48323.011</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -8032,7 +8020,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
       <c r="B5" t="n">
@@ -8048,7 +8036,7 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>60711.985</v>
+        <v>12535.341</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -8066,10 +8054,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>71937.889</v>
+        <v>35640.824</v>
       </c>
       <c r="M5" t="n">
-        <v>83448.56</v>
+        <v>51264.145</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -8178,7 +8166,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
       <c r="B6" t="n">
@@ -8197,7 +8185,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>69274.144</v>
+        <v>28346.784</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -8212,10 +8200,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>69291.52499999999</v>
+        <v>28640.457</v>
       </c>
       <c r="M6" t="n">
-        <v>77116.255</v>
+        <v>43395.716</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
@@ -8324,7 +8312,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
       <c r="B7" t="n">
@@ -8346,7 +8334,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>61676.846</v>
+        <v>15506.144</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -8361,10 +8349,10 @@
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>71817.85000000001</v>
+        <v>29493.358</v>
       </c>
       <c r="N7" t="n">
-        <v>64756.808</v>
+        <v>21685.058</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
@@ -8470,7 +8458,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>7</v>
       </c>
       <c r="B8" t="n">
@@ -8489,13 +8477,13 @@
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>57216.709</v>
+        <v>14564.55</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>61433.651</v>
+        <v>18185.227</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -8510,16 +8498,16 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>65195.117</v>
+        <v>25250.586</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>75795.01700000001</v>
+        <v>38270.479</v>
       </c>
       <c r="Q8" t="n">
-        <v>79682.951</v>
+        <v>53404.882</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -8616,7 +8604,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>8</v>
       </c>
       <c r="B9" t="n">
@@ -8638,13 +8626,13 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>57704.864</v>
+        <v>17178.186</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>62591.365</v>
+        <v>23384.789</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -8656,16 +8644,16 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>67746.727</v>
+        <v>31055.636</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>75930.70699999999</v>
+        <v>43114.937</v>
       </c>
       <c r="Q9" t="n">
-        <v>75073.77099999999</v>
+        <v>45951.332</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
@@ -8762,7 +8750,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>9</v>
       </c>
       <c r="B10" t="n">
@@ -8787,13 +8775,13 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>59057.218</v>
+        <v>22152.279</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>86060.952</v>
+        <v>58172.093</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -8808,10 +8796,10 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>82233.91099999999</v>
+        <v>51575.493</v>
       </c>
       <c r="Q10" t="n">
-        <v>72705.19500000001</v>
+        <v>38819.037</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
@@ -8823,10 +8811,10 @@
         <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>84217.42</v>
+        <v>66445.243</v>
       </c>
       <c r="V10" t="n">
-        <v>97501.91499999999</v>
+        <v>81208.442</v>
       </c>
       <c r="W10" t="n">
         <v>0</v>
@@ -8908,7 +8896,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>10</v>
       </c>
       <c r="B11" t="n">
@@ -8936,7 +8924,7 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>78134.395</v>
+        <v>54737.557</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -8972,7 +8960,7 @@
         <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>88312.428</v>
+        <v>78718.607</v>
       </c>
       <c r="W11" t="n">
         <v>0</v>
@@ -9054,7 +9042,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" t="n">
         <v>11</v>
       </c>
       <c r="B12" t="n">
@@ -9091,7 +9079,7 @@
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>68684.101</v>
+        <v>22476.43</v>
       </c>
       <c r="N12" t="n">
         <v>0</v>
@@ -9106,10 +9094,10 @@
         <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>67653.79399999999</v>
+        <v>25219.737</v>
       </c>
       <c r="S12" t="n">
-        <v>72321.107</v>
+        <v>31118.837</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -9200,7 +9188,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" t="n">
         <v>12</v>
       </c>
       <c r="B13" t="n">
@@ -9219,7 +9207,7 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>63231.839</v>
+        <v>26931.207</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -9243,7 +9231,7 @@
         <v>0</v>
       </c>
       <c r="O13" t="n">
-        <v>66552.51700000001</v>
+        <v>11027.348</v>
       </c>
       <c r="P13" t="n">
         <v>0</v>
@@ -9255,7 +9243,7 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>69669.44500000001</v>
+        <v>25259.654</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -9346,7 +9334,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="n">
         <v>13</v>
       </c>
       <c r="B14" t="n">
@@ -9368,7 +9356,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>59590.708</v>
+        <v>23503.107</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -9389,10 +9377,10 @@
         <v>0</v>
       </c>
       <c r="O14" t="n">
-        <v>67652.83500000001</v>
+        <v>15548.88</v>
       </c>
       <c r="P14" t="n">
-        <v>68268.784</v>
+        <v>17269.127</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
@@ -9492,7 +9480,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" t="n">
         <v>14</v>
       </c>
       <c r="B15" t="n">
@@ -9532,13 +9520,13 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>57119.365</v>
+        <v>13941.468</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>65123.7</v>
+        <v>8396.468999999999</v>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
@@ -9550,7 +9538,7 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>71297.33500000001</v>
+        <v>29635.784</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -9562,7 +9550,7 @@
         <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>90821.374</v>
+        <v>80714.239</v>
       </c>
       <c r="Y15" t="n">
         <v>0</v>
@@ -9638,7 +9626,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" t="n">
         <v>15</v>
       </c>
       <c r="B16" t="n">
@@ -9687,7 +9675,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>69429.914</v>
+        <v>35535.388</v>
       </c>
       <c r="R16" t="n">
         <v>0</v>
@@ -9699,7 +9687,7 @@
         <v>0</v>
       </c>
       <c r="U16" t="n">
-        <v>84236.71000000001</v>
+        <v>57439.085</v>
       </c>
       <c r="V16" t="n">
         <v>0</v>
@@ -9708,7 +9696,7 @@
         <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>83377.682</v>
+        <v>75206.954</v>
       </c>
       <c r="Y16" t="n">
         <v>0</v>
@@ -9784,7 +9772,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" t="n">
         <v>16</v>
       </c>
       <c r="B17" t="n">
@@ -9845,7 +9833,7 @@
         <v>0</v>
       </c>
       <c r="U17" t="n">
-        <v>66825.833</v>
+        <v>30067.019</v>
       </c>
       <c r="V17" t="n">
         <v>0</v>
@@ -9930,7 +9918,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" t="n">
         <v>17</v>
       </c>
       <c r="B18" t="n">
@@ -9985,7 +9973,7 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>66662.33</v>
+        <v>20700.009</v>
       </c>
       <c r="T18" t="n">
         <v>0</v>
@@ -10066,7 +10054,7 @@
         <v>0</v>
       </c>
       <c r="AT18" t="n">
-        <v>66817.18700000001</v>
+        <v>22941.296</v>
       </c>
       <c r="AU18" t="n">
         <v>0</v>
@@ -10076,7 +10064,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" t="n">
         <v>18</v>
       </c>
       <c r="B19" t="n">
@@ -10113,13 +10101,13 @@
         <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>59342.879</v>
+        <v>22769.993</v>
       </c>
       <c r="N19" t="n">
         <v>0</v>
       </c>
       <c r="O19" t="n">
-        <v>69463.68399999999</v>
+        <v>26319.681</v>
       </c>
       <c r="P19" t="n">
         <v>0</v>
@@ -10134,7 +10122,7 @@
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>64449.096</v>
+        <v>12795.93</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
@@ -10212,7 +10200,7 @@
         <v>0</v>
       </c>
       <c r="AT19" t="n">
-        <v>65120.563</v>
+        <v>17642.05</v>
       </c>
       <c r="AU19" t="n">
         <v>0</v>
@@ -10222,7 +10210,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" t="n">
         <v>19</v>
       </c>
       <c r="B20" t="n">
@@ -10265,7 +10253,7 @@
         <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>62323.257</v>
+        <v>27442.088</v>
       </c>
       <c r="P20" t="n">
         <v>0</v>
@@ -10277,22 +10265,22 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>55973.158</v>
+        <v>11697.556</v>
       </c>
       <c r="T20" t="n">
         <v>0</v>
       </c>
       <c r="U20" t="n">
-        <v>85630.205</v>
+        <v>64220.296</v>
       </c>
       <c r="V20" t="n">
         <v>0</v>
       </c>
       <c r="W20" t="n">
-        <v>72546.46400000001</v>
+        <v>36628.953</v>
       </c>
       <c r="X20" t="n">
-        <v>80893.908</v>
+        <v>48775.69</v>
       </c>
       <c r="Y20" t="n">
         <v>0</v>
@@ -10368,7 +10356,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" t="n">
         <v>20</v>
       </c>
       <c r="B21" t="n">
@@ -10438,16 +10426,16 @@
         <v>0</v>
       </c>
       <c r="X21" t="n">
-        <v>84829.58500000001</v>
+        <v>63288.981</v>
       </c>
       <c r="Y21" t="n">
         <v>0</v>
       </c>
       <c r="Z21" t="n">
-        <v>81634.947</v>
+        <v>54972.885</v>
       </c>
       <c r="AA21" t="n">
-        <v>107122.453</v>
+        <v>111329.769</v>
       </c>
       <c r="AB21" t="n">
         <v>0</v>
@@ -10501,7 +10489,7 @@
         <v>0</v>
       </c>
       <c r="AS21" t="n">
-        <v>88385.481</v>
+        <v>79366.30899999999</v>
       </c>
       <c r="AT21" t="n">
         <v>0</v>
@@ -10514,7 +10502,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" t="n">
         <v>21</v>
       </c>
       <c r="B22" t="n">
@@ -10575,7 +10563,7 @@
         <v>0</v>
       </c>
       <c r="U22" t="n">
-        <v>64869.357</v>
+        <v>24379.466</v>
       </c>
       <c r="V22" t="n">
         <v>0</v>
@@ -10590,7 +10578,7 @@
         <v>0</v>
       </c>
       <c r="Z22" t="n">
-        <v>76326.61199999999</v>
+        <v>42789.519</v>
       </c>
       <c r="AA22" t="n">
         <v>0</v>
@@ -10660,7 +10648,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" t="n">
         <v>22</v>
       </c>
       <c r="B23" t="n">
@@ -10718,10 +10706,10 @@
         <v>0</v>
       </c>
       <c r="T23" t="n">
-        <v>63833.163</v>
+        <v>33943.576</v>
       </c>
       <c r="U23" t="n">
-        <v>91349.469</v>
+        <v>84430.912</v>
       </c>
       <c r="V23" t="n">
         <v>0</v>
@@ -10730,7 +10718,7 @@
         <v>0</v>
       </c>
       <c r="X23" t="n">
-        <v>70463.61599999999</v>
+        <v>27769.232</v>
       </c>
       <c r="Y23" t="n">
         <v>0</v>
@@ -10806,7 +10794,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" t="n">
         <v>23</v>
       </c>
       <c r="B24" t="n">
@@ -10867,7 +10855,7 @@
         <v>0</v>
       </c>
       <c r="U24" t="n">
-        <v>79526.45299999999</v>
+        <v>59812.492</v>
       </c>
       <c r="V24" t="n">
         <v>0</v>
@@ -10879,7 +10867,7 @@
         <v>0</v>
       </c>
       <c r="Y24" t="n">
-        <v>63593.494</v>
+        <v>10959.301</v>
       </c>
       <c r="Z24" t="n">
         <v>0</v>
@@ -10945,14 +10933,14 @@
         <v>0</v>
       </c>
       <c r="AU24" t="n">
-        <v>62356.352</v>
+        <v>12061.556</v>
       </c>
       <c r="AV24" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" t="n">
         <v>24</v>
       </c>
       <c r="B25" t="n">
@@ -11022,7 +11010,7 @@
         <v>0</v>
       </c>
       <c r="X25" t="n">
-        <v>55627.749</v>
+        <v>10023.696</v>
       </c>
       <c r="Y25" t="n">
         <v>0</v>
@@ -11031,7 +11019,7 @@
         <v>0</v>
       </c>
       <c r="AA25" t="n">
-        <v>84975.463</v>
+        <v>57140.942</v>
       </c>
       <c r="AB25" t="n">
         <v>0</v>
@@ -11091,14 +11079,14 @@
         <v>0</v>
       </c>
       <c r="AU25" t="n">
-        <v>62180.441</v>
+        <v>7026.85</v>
       </c>
       <c r="AV25" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" t="n">
         <v>25</v>
       </c>
       <c r="B26" t="n">
@@ -11180,13 +11168,13 @@
         <v>0</v>
       </c>
       <c r="AB26" t="n">
-        <v>79424.235</v>
+        <v>49859.744</v>
       </c>
       <c r="AC26" t="n">
         <v>0</v>
       </c>
       <c r="AD26" t="n">
-        <v>101761.957</v>
+        <v>94382.253</v>
       </c>
       <c r="AE26" t="n">
         <v>0</v>
@@ -11231,7 +11219,7 @@
         <v>0</v>
       </c>
       <c r="AS26" t="n">
-        <v>63898.503</v>
+        <v>25655.797</v>
       </c>
       <c r="AT26" t="n">
         <v>0</v>
@@ -11244,7 +11232,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" t="n">
         <v>26</v>
       </c>
       <c r="B27" t="n">
@@ -11326,19 +11314,19 @@
         <v>0</v>
       </c>
       <c r="AB27" t="n">
-        <v>94695.545</v>
+        <v>80828.85400000001</v>
       </c>
       <c r="AC27" t="n">
         <v>0</v>
       </c>
       <c r="AD27" t="n">
-        <v>85873.183</v>
+        <v>76645.742</v>
       </c>
       <c r="AE27" t="n">
-        <v>102611.209</v>
+        <v>102079.686</v>
       </c>
       <c r="AF27" t="n">
-        <v>83890.12699999999</v>
+        <v>57774.722</v>
       </c>
       <c r="AG27" t="n">
         <v>0</v>
@@ -11347,7 +11335,7 @@
         <v>0</v>
       </c>
       <c r="AI27" t="n">
-        <v>85071.546</v>
+        <v>67748.359</v>
       </c>
       <c r="AJ27" t="n">
         <v>0</v>
@@ -11377,7 +11365,7 @@
         <v>0</v>
       </c>
       <c r="AS27" t="n">
-        <v>83638.268</v>
+        <v>58555.131</v>
       </c>
       <c r="AT27" t="n">
         <v>0</v>
@@ -11390,7 +11378,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" t="n">
         <v>27</v>
       </c>
       <c r="B28" t="n">
@@ -11469,7 +11457,7 @@
         <v>0</v>
       </c>
       <c r="AA28" t="n">
-        <v>89174.75199999999</v>
+        <v>76483.664</v>
       </c>
       <c r="AB28" t="n">
         <v>0</v>
@@ -11478,10 +11466,10 @@
         <v>0</v>
       </c>
       <c r="AD28" t="n">
-        <v>79087.192</v>
+        <v>52652.261</v>
       </c>
       <c r="AE28" t="n">
-        <v>74350.798</v>
+        <v>42644.701</v>
       </c>
       <c r="AF28" t="n">
         <v>0</v>
@@ -11536,7 +11524,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" t="n">
         <v>28</v>
       </c>
       <c r="B29" t="n">
@@ -11615,7 +11603,7 @@
         <v>0</v>
       </c>
       <c r="AA29" t="n">
-        <v>118965.559</v>
+        <v>121861.008</v>
       </c>
       <c r="AB29" t="n">
         <v>0</v>
@@ -11633,13 +11621,13 @@
         <v>0</v>
       </c>
       <c r="AG29" t="n">
-        <v>107551.425</v>
+        <v>106795.513</v>
       </c>
       <c r="AH29" t="n">
-        <v>99000.243</v>
+        <v>81963.177</v>
       </c>
       <c r="AI29" t="n">
-        <v>121415.432</v>
+        <v>127171.671</v>
       </c>
       <c r="AJ29" t="n">
         <v>0</v>
@@ -11682,7 +11670,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" t="n">
         <v>29</v>
       </c>
       <c r="B30" t="n">
@@ -11773,7 +11761,7 @@
         <v>0</v>
       </c>
       <c r="AE30" t="n">
-        <v>72907.624</v>
+        <v>39066.869</v>
       </c>
       <c r="AF30" t="n">
         <v>0</v>
@@ -11788,13 +11776,13 @@
         <v>0</v>
       </c>
       <c r="AJ30" t="n">
-        <v>95550.784</v>
+        <v>83111.54300000001</v>
       </c>
       <c r="AK30" t="n">
         <v>0</v>
       </c>
       <c r="AL30" t="n">
-        <v>85841.454</v>
+        <v>77129.147</v>
       </c>
       <c r="AM30" t="n">
         <v>0</v>
@@ -11828,7 +11816,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" t="n">
         <v>30</v>
       </c>
       <c r="B31" t="n">
@@ -11916,7 +11904,7 @@
         <v>0</v>
       </c>
       <c r="AD31" t="n">
-        <v>68585.444</v>
+        <v>36986.538</v>
       </c>
       <c r="AE31" t="n">
         <v>0</v>
@@ -11934,13 +11922,13 @@
         <v>0</v>
       </c>
       <c r="AJ31" t="n">
-        <v>84203.257</v>
+        <v>61789.812</v>
       </c>
       <c r="AK31" t="n">
         <v>0</v>
       </c>
       <c r="AL31" t="n">
-        <v>83434.887</v>
+        <v>60944.277</v>
       </c>
       <c r="AM31" t="n">
         <v>0</v>
@@ -11974,7 +11962,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" t="n">
         <v>31</v>
       </c>
       <c r="B32" t="n">
@@ -12077,7 +12065,7 @@
         <v>0</v>
       </c>
       <c r="AI32" t="n">
-        <v>64850.377</v>
+        <v>23912.606</v>
       </c>
       <c r="AJ32" t="n">
         <v>0</v>
@@ -12086,7 +12074,7 @@
         <v>0</v>
       </c>
       <c r="AL32" t="n">
-        <v>100934.794</v>
+        <v>100117.747</v>
       </c>
       <c r="AM32" t="n">
         <v>0</v>
@@ -12120,7 +12108,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" t="n">
         <v>32</v>
       </c>
       <c r="B33" t="n">
@@ -12199,7 +12187,7 @@
         <v>0</v>
       </c>
       <c r="AA33" t="n">
-        <v>69954.36599999999</v>
+        <v>26939.691</v>
       </c>
       <c r="AB33" t="n">
         <v>0</v>
@@ -12266,7 +12254,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" t="n">
         <v>33</v>
       </c>
       <c r="B34" t="n">
@@ -12369,19 +12357,19 @@
         <v>0</v>
       </c>
       <c r="AI34" t="n">
-        <v>83086.13499999999</v>
+        <v>52917.19</v>
       </c>
       <c r="AJ34" t="n">
         <v>0</v>
       </c>
       <c r="AK34" t="n">
-        <v>67961.99000000001</v>
+        <v>26774.788</v>
       </c>
       <c r="AL34" t="n">
         <v>0</v>
       </c>
       <c r="AM34" t="n">
-        <v>74952.629</v>
+        <v>47991.331</v>
       </c>
       <c r="AN34" t="n">
         <v>0</v>
@@ -12412,7 +12400,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" t="n">
         <v>34</v>
       </c>
       <c r="B35" t="n">
@@ -12506,7 +12494,7 @@
         <v>0</v>
       </c>
       <c r="AF35" t="n">
-        <v>59098.79</v>
+        <v>22277.779</v>
       </c>
       <c r="AG35" t="n">
         <v>0</v>
@@ -12527,7 +12515,7 @@
         <v>0</v>
       </c>
       <c r="AM35" t="n">
-        <v>62730.815</v>
+        <v>25536.107</v>
       </c>
       <c r="AN35" t="n">
         <v>0</v>
@@ -12558,7 +12546,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" t="n">
         <v>35</v>
       </c>
       <c r="B36" t="n">
@@ -12670,7 +12658,7 @@
         <v>0</v>
       </c>
       <c r="AL36" t="n">
-        <v>62165.115</v>
+        <v>22105.039</v>
       </c>
       <c r="AM36" t="n">
         <v>0</v>
@@ -12704,7 +12692,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" t="n">
         <v>36</v>
       </c>
       <c r="B37" t="n">
@@ -12804,10 +12792,10 @@
         <v>0</v>
       </c>
       <c r="AH37" t="n">
-        <v>62233.913</v>
+        <v>25045.029</v>
       </c>
       <c r="AI37" t="n">
-        <v>82484.583</v>
+        <v>52961.418</v>
       </c>
       <c r="AJ37" t="n">
         <v>0</v>
@@ -12819,7 +12807,7 @@
         <v>0</v>
       </c>
       <c r="AM37" t="n">
-        <v>67865.70299999999</v>
+        <v>37191.118</v>
       </c>
       <c r="AN37" t="n">
         <v>0</v>
@@ -12850,7 +12838,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" t="n">
         <v>37</v>
       </c>
       <c r="B38" t="n">
@@ -12977,7 +12965,7 @@
         <v>0</v>
       </c>
       <c r="AQ38" t="n">
-        <v>61726.388</v>
+        <v>18801.124</v>
       </c>
       <c r="AR38" t="n">
         <v>0</v>
@@ -12996,7 +12984,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" t="n">
         <v>38</v>
       </c>
       <c r="B39" t="n">
@@ -13099,7 +13087,7 @@
         <v>0</v>
       </c>
       <c r="AI39" t="n">
-        <v>62730.815</v>
+        <v>25536.107</v>
       </c>
       <c r="AJ39" t="n">
         <v>0</v>
@@ -13142,7 +13130,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" t="n">
         <v>39</v>
       </c>
       <c r="B40" t="n">
@@ -13251,13 +13239,13 @@
         <v>0</v>
       </c>
       <c r="AK40" t="n">
-        <v>82730.30100000001</v>
+        <v>54068.701</v>
       </c>
       <c r="AL40" t="n">
         <v>0</v>
       </c>
       <c r="AM40" t="n">
-        <v>92704.552</v>
+        <v>83344.196</v>
       </c>
       <c r="AN40" t="n">
         <v>0</v>
@@ -13288,7 +13276,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" t="n">
         <v>40</v>
       </c>
       <c r="B41" t="n">
@@ -13400,7 +13388,7 @@
         <v>0</v>
       </c>
       <c r="AL41" t="n">
-        <v>84001.08500000001</v>
+        <v>57997.797</v>
       </c>
       <c r="AM41" t="n">
         <v>0</v>
@@ -13434,7 +13422,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" t="n">
         <v>41</v>
       </c>
       <c r="B42" t="n">
@@ -13543,13 +13531,13 @@
         <v>0</v>
       </c>
       <c r="AK42" t="n">
-        <v>118644.816</v>
+        <v>128136.207</v>
       </c>
       <c r="AL42" t="n">
         <v>0</v>
       </c>
       <c r="AM42" t="n">
-        <v>116659.859</v>
+        <v>132479.058</v>
       </c>
       <c r="AN42" t="n">
         <v>0</v>
@@ -13580,7 +13568,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" t="n">
         <v>42</v>
       </c>
       <c r="B43" t="n">
@@ -13726,7 +13714,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" t="n">
         <v>43</v>
       </c>
       <c r="B44" t="n">
@@ -13872,7 +13860,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" t="n">
         <v>44</v>
       </c>
       <c r="B45" t="n">
@@ -13948,19 +13936,19 @@
         <v>0</v>
       </c>
       <c r="Z45" t="n">
-        <v>59993.223</v>
+        <v>24235.769</v>
       </c>
       <c r="AA45" t="n">
         <v>0</v>
       </c>
       <c r="AB45" t="n">
-        <v>72183.13</v>
+        <v>39223.15</v>
       </c>
       <c r="AC45" t="n">
         <v>0</v>
       </c>
       <c r="AD45" t="n">
-        <v>88018.28200000001</v>
+        <v>79265.137</v>
       </c>
       <c r="AE45" t="n">
         <v>0</v>
@@ -14018,7 +14006,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" t="n">
         <v>45</v>
       </c>
       <c r="B46" t="n">
@@ -14073,10 +14061,10 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>57300.73</v>
+        <v>16314.371</v>
       </c>
       <c r="T46" t="n">
-        <v>57832.78</v>
+        <v>17653.422</v>
       </c>
       <c r="U46" t="n">
         <v>0</v>
@@ -14085,10 +14073,10 @@
         <v>0</v>
       </c>
       <c r="W46" t="n">
-        <v>62754.984</v>
+        <v>32624.793</v>
       </c>
       <c r="X46" t="n">
-        <v>76533.738</v>
+        <v>51875.313</v>
       </c>
       <c r="Y46" t="n">
         <v>0</v>
@@ -14164,7 +14152,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" t="n">
         <v>46</v>
       </c>
       <c r="B47" t="n">
@@ -14237,13 +14225,13 @@
         <v>0</v>
       </c>
       <c r="Y47" t="n">
-        <v>53339.219</v>
+        <v>6464.535</v>
       </c>
       <c r="Z47" t="n">
-        <v>78622.86199999999</v>
+        <v>62768.97</v>
       </c>
       <c r="AA47" t="n">
-        <v>84319.22500000001</v>
+        <v>56735.007</v>
       </c>
       <c r="AB47" t="n">
         <v>0</v>
@@ -14297,7 +14285,7 @@
         <v>0</v>
       </c>
       <c r="AS47" t="n">
-        <v>83299.246</v>
+        <v>60230.576</v>
       </c>
       <c r="AT47" t="n">
         <v>0</v>
@@ -14310,14 +14298,14 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" t="n">
         <v>47</v>
       </c>
       <c r="B48" t="n">
         <v>0</v>
       </c>
       <c r="C48" t="n">
-        <v>65103.006</v>
+        <v>16163.714</v>
       </c>
       <c r="D48" t="n">
         <v>0</v>
@@ -14341,7 +14329,7 @@
         <v>0</v>
       </c>
       <c r="K48" t="n">
-        <v>118239.547</v>
+        <v>122328.424</v>
       </c>
       <c r="L48" t="n">
         <v>0</v>
@@ -14470,150 +14458,150 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="n">
+      <c r="B1" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="n">
+      <c r="C1" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="n">
+      <c r="D1" t="n">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="n">
+      <c r="E1" t="n">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="n">
+      <c r="F1" t="n">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="n">
+      <c r="G1" t="n">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="n">
+      <c r="H1" t="n">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="n">
+      <c r="I1" t="n">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="n">
+      <c r="J1" t="n">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="n">
+      <c r="K1" t="n">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="n">
+      <c r="L1" t="n">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="n">
+      <c r="M1" t="n">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="n">
+      <c r="N1" t="n">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="n">
+      <c r="O1" t="n">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="n">
+      <c r="P1" t="n">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="n">
+      <c r="Q1" t="n">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="n">
+      <c r="R1" t="n">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="n">
+      <c r="S1" t="n">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="n">
+      <c r="T1" t="n">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="n">
+      <c r="U1" t="n">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="n">
+      <c r="V1" t="n">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="n">
+      <c r="W1" t="n">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="n">
+      <c r="X1" t="n">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="n">
+      <c r="Y1" t="n">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="n">
+      <c r="Z1" t="n">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="n">
+      <c r="AA1" t="n">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="n">
+      <c r="AB1" t="n">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="n">
+      <c r="AC1" t="n">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="n">
+      <c r="AD1" t="n">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="n">
+      <c r="AE1" t="n">
         <v>30</v>
       </c>
-      <c r="AF1" s="1" t="n">
+      <c r="AF1" t="n">
         <v>31</v>
       </c>
-      <c r="AG1" s="1" t="n">
+      <c r="AG1" t="n">
         <v>32</v>
       </c>
-      <c r="AH1" s="1" t="n">
+      <c r="AH1" t="n">
         <v>33</v>
       </c>
-      <c r="AI1" s="1" t="n">
+      <c r="AI1" t="n">
         <v>34</v>
       </c>
-      <c r="AJ1" s="1" t="n">
+      <c r="AJ1" t="n">
         <v>35</v>
       </c>
-      <c r="AK1" s="1" t="n">
+      <c r="AK1" t="n">
         <v>36</v>
       </c>
-      <c r="AL1" s="1" t="n">
+      <c r="AL1" t="n">
         <v>37</v>
       </c>
-      <c r="AM1" s="1" t="n">
+      <c r="AM1" t="n">
         <v>38</v>
       </c>
-      <c r="AN1" s="1" t="n">
+      <c r="AN1" t="n">
         <v>39</v>
       </c>
-      <c r="AO1" s="1" t="n">
+      <c r="AO1" t="n">
         <v>40</v>
       </c>
-      <c r="AP1" s="1" t="n">
+      <c r="AP1" t="n">
         <v>41</v>
       </c>
-      <c r="AQ1" s="1" t="n">
+      <c r="AQ1" t="n">
         <v>42</v>
       </c>
-      <c r="AR1" s="1" t="n">
+      <c r="AR1" t="n">
         <v>43</v>
       </c>
-      <c r="AS1" s="1" t="n">
+      <c r="AS1" t="n">
         <v>44</v>
       </c>
-      <c r="AT1" s="1" t="n">
+      <c r="AT1" t="n">
         <v>45</v>
       </c>
-      <c r="AU1" s="1" t="n">
+      <c r="AU1" t="n">
         <v>46</v>
       </c>
-      <c r="AV1" s="1" t="n">
+      <c r="AV1" t="n">
         <v>47</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="n">
@@ -14759,7 +14747,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
       <c r="B3" t="n">
@@ -14905,7 +14893,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
       <c r="B4" t="n">
@@ -15051,7 +15039,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
       <c r="B5" t="n">
@@ -15197,7 +15185,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
       <c r="B6" t="n">
@@ -15343,7 +15331,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
       <c r="B7" t="n">
@@ -15489,7 +15477,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>7</v>
       </c>
       <c r="B8" t="n">
@@ -15635,7 +15623,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>8</v>
       </c>
       <c r="B9" t="n">
@@ -15781,7 +15769,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>9</v>
       </c>
       <c r="B10" t="n">
@@ -15927,7 +15915,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>10</v>
       </c>
       <c r="B11" t="n">
@@ -16073,7 +16061,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" t="n">
         <v>11</v>
       </c>
       <c r="B12" t="n">
@@ -16219,7 +16207,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" t="n">
         <v>12</v>
       </c>
       <c r="B13" t="n">
@@ -16365,7 +16353,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="n">
         <v>13</v>
       </c>
       <c r="B14" t="n">
@@ -16511,7 +16499,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" t="n">
         <v>14</v>
       </c>
       <c r="B15" t="n">
@@ -16657,7 +16645,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" t="n">
         <v>15</v>
       </c>
       <c r="B16" t="n">
@@ -16803,7 +16791,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" t="n">
         <v>16</v>
       </c>
       <c r="B17" t="n">
@@ -16949,7 +16937,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" t="n">
         <v>17</v>
       </c>
       <c r="B18" t="n">
@@ -17095,7 +17083,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" t="n">
         <v>18</v>
       </c>
       <c r="B19" t="n">
@@ -17241,7 +17229,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" t="n">
         <v>19</v>
       </c>
       <c r="B20" t="n">
@@ -17387,7 +17375,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" t="n">
         <v>20</v>
       </c>
       <c r="B21" t="n">
@@ -17533,7 +17521,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" t="n">
         <v>21</v>
       </c>
       <c r="B22" t="n">
@@ -17679,7 +17667,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" t="n">
         <v>22</v>
       </c>
       <c r="B23" t="n">
@@ -17825,7 +17813,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" t="n">
         <v>23</v>
       </c>
       <c r="B24" t="n">
@@ -17971,7 +17959,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" t="n">
         <v>24</v>
       </c>
       <c r="B25" t="n">
@@ -18117,7 +18105,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" t="n">
         <v>25</v>
       </c>
       <c r="B26" t="n">
@@ -18263,7 +18251,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" t="n">
         <v>26</v>
       </c>
       <c r="B27" t="n">
@@ -18409,7 +18397,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" t="n">
         <v>27</v>
       </c>
       <c r="B28" t="n">
@@ -18555,7 +18543,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" t="n">
         <v>28</v>
       </c>
       <c r="B29" t="n">
@@ -18701,7 +18689,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" t="n">
         <v>29</v>
       </c>
       <c r="B30" t="n">
@@ -18847,7 +18835,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" t="n">
         <v>30</v>
       </c>
       <c r="B31" t="n">
@@ -18993,7 +18981,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" t="n">
         <v>31</v>
       </c>
       <c r="B32" t="n">
@@ -19139,7 +19127,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" t="n">
         <v>32</v>
       </c>
       <c r="B33" t="n">
@@ -19285,7 +19273,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" t="n">
         <v>33</v>
       </c>
       <c r="B34" t="n">
@@ -19431,7 +19419,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" t="n">
         <v>34</v>
       </c>
       <c r="B35" t="n">
@@ -19577,7 +19565,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" t="n">
         <v>35</v>
       </c>
       <c r="B36" t="n">
@@ -19723,7 +19711,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" t="n">
         <v>36</v>
       </c>
       <c r="B37" t="n">
@@ -19869,7 +19857,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" t="n">
         <v>37</v>
       </c>
       <c r="B38" t="n">
@@ -20015,7 +20003,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" t="n">
         <v>38</v>
       </c>
       <c r="B39" t="n">
@@ -20161,7 +20149,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" t="n">
         <v>39</v>
       </c>
       <c r="B40" t="n">
@@ -20307,7 +20295,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" t="n">
         <v>40</v>
       </c>
       <c r="B41" t="n">
@@ -20453,7 +20441,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" t="n">
         <v>41</v>
       </c>
       <c r="B42" t="n">
@@ -20599,7 +20587,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" t="n">
         <v>42</v>
       </c>
       <c r="B43" t="n">
@@ -20745,7 +20733,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" t="n">
         <v>43</v>
       </c>
       <c r="B44" t="n">
@@ -20891,7 +20879,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" t="n">
         <v>44</v>
       </c>
       <c r="B45" t="n">
@@ -21037,7 +21025,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" t="n">
         <v>45</v>
       </c>
       <c r="B46" t="n">
@@ -21183,7 +21171,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" t="n">
         <v>46</v>
       </c>
       <c r="B47" t="n">
@@ -21329,7 +21317,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" t="n">
         <v>47</v>
       </c>
       <c r="B48" t="n">
@@ -21489,150 +21477,150 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="n">
+      <c r="B1" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="n">
+      <c r="C1" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="n">
+      <c r="D1" t="n">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="n">
+      <c r="E1" t="n">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="n">
+      <c r="F1" t="n">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="n">
+      <c r="G1" t="n">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="n">
+      <c r="H1" t="n">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="n">
+      <c r="I1" t="n">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="n">
+      <c r="J1" t="n">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="n">
+      <c r="K1" t="n">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="n">
+      <c r="L1" t="n">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="n">
+      <c r="M1" t="n">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="n">
+      <c r="N1" t="n">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="n">
+      <c r="O1" t="n">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="n">
+      <c r="P1" t="n">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="n">
+      <c r="Q1" t="n">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="n">
+      <c r="R1" t="n">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="n">
+      <c r="S1" t="n">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="n">
+      <c r="T1" t="n">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="n">
+      <c r="U1" t="n">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="n">
+      <c r="V1" t="n">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="n">
+      <c r="W1" t="n">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="n">
+      <c r="X1" t="n">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="n">
+      <c r="Y1" t="n">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="n">
+      <c r="Z1" t="n">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="n">
+      <c r="AA1" t="n">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="n">
+      <c r="AB1" t="n">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="n">
+      <c r="AC1" t="n">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="n">
+      <c r="AD1" t="n">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="n">
+      <c r="AE1" t="n">
         <v>30</v>
       </c>
-      <c r="AF1" s="1" t="n">
+      <c r="AF1" t="n">
         <v>31</v>
       </c>
-      <c r="AG1" s="1" t="n">
+      <c r="AG1" t="n">
         <v>32</v>
       </c>
-      <c r="AH1" s="1" t="n">
+      <c r="AH1" t="n">
         <v>33</v>
       </c>
-      <c r="AI1" s="1" t="n">
+      <c r="AI1" t="n">
         <v>34</v>
       </c>
-      <c r="AJ1" s="1" t="n">
+      <c r="AJ1" t="n">
         <v>35</v>
       </c>
-      <c r="AK1" s="1" t="n">
+      <c r="AK1" t="n">
         <v>36</v>
       </c>
-      <c r="AL1" s="1" t="n">
+      <c r="AL1" t="n">
         <v>37</v>
       </c>
-      <c r="AM1" s="1" t="n">
+      <c r="AM1" t="n">
         <v>38</v>
       </c>
-      <c r="AN1" s="1" t="n">
+      <c r="AN1" t="n">
         <v>39</v>
       </c>
-      <c r="AO1" s="1" t="n">
+      <c r="AO1" t="n">
         <v>40</v>
       </c>
-      <c r="AP1" s="1" t="n">
+      <c r="AP1" t="n">
         <v>41</v>
       </c>
-      <c r="AQ1" s="1" t="n">
+      <c r="AQ1" t="n">
         <v>42</v>
       </c>
-      <c r="AR1" s="1" t="n">
+      <c r="AR1" t="n">
         <v>43</v>
       </c>
-      <c r="AS1" s="1" t="n">
+      <c r="AS1" t="n">
         <v>44</v>
       </c>
-      <c r="AT1" s="1" t="n">
+      <c r="AT1" t="n">
         <v>45</v>
       </c>
-      <c r="AU1" s="1" t="n">
+      <c r="AU1" t="n">
         <v>46</v>
       </c>
-      <c r="AV1" s="1" t="n">
+      <c r="AV1" t="n">
         <v>47</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="n">
@@ -21778,7 +21766,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
       <c r="B3" t="n">
@@ -21924,7 +21912,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
       <c r="B4" t="n">
@@ -22070,7 +22058,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
       <c r="B5" t="n">
@@ -22216,7 +22204,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
       <c r="B6" t="n">
@@ -22362,7 +22350,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
       <c r="B7" t="n">
@@ -22508,7 +22496,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>7</v>
       </c>
       <c r="B8" t="n">
@@ -22654,7 +22642,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>8</v>
       </c>
       <c r="B9" t="n">
@@ -22800,7 +22788,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>9</v>
       </c>
       <c r="B10" t="n">
@@ -22946,7 +22934,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>10</v>
       </c>
       <c r="B11" t="n">
@@ -23092,7 +23080,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" t="n">
         <v>11</v>
       </c>
       <c r="B12" t="n">
@@ -23238,7 +23226,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" t="n">
         <v>12</v>
       </c>
       <c r="B13" t="n">
@@ -23384,7 +23372,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="n">
         <v>13</v>
       </c>
       <c r="B14" t="n">
@@ -23530,7 +23518,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" t="n">
         <v>14</v>
       </c>
       <c r="B15" t="n">
@@ -23676,7 +23664,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" t="n">
         <v>15</v>
       </c>
       <c r="B16" t="n">
@@ -23822,7 +23810,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" t="n">
         <v>16</v>
       </c>
       <c r="B17" t="n">
@@ -23968,7 +23956,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" t="n">
         <v>17</v>
       </c>
       <c r="B18" t="n">
@@ -24114,7 +24102,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" t="n">
         <v>18</v>
       </c>
       <c r="B19" t="n">
@@ -24260,7 +24248,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" t="n">
         <v>19</v>
       </c>
       <c r="B20" t="n">
@@ -24406,7 +24394,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" t="n">
         <v>20</v>
       </c>
       <c r="B21" t="n">
@@ -24552,7 +24540,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" t="n">
         <v>21</v>
       </c>
       <c r="B22" t="n">
@@ -24698,7 +24686,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" t="n">
         <v>22</v>
       </c>
       <c r="B23" t="n">
@@ -24844,7 +24832,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" t="n">
         <v>23</v>
       </c>
       <c r="B24" t="n">
@@ -24990,7 +24978,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" t="n">
         <v>24</v>
       </c>
       <c r="B25" t="n">
@@ -25136,7 +25124,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" t="n">
         <v>25</v>
       </c>
       <c r="B26" t="n">
@@ -25282,7 +25270,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" t="n">
         <v>26</v>
       </c>
       <c r="B27" t="n">
@@ -25428,7 +25416,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" t="n">
         <v>27</v>
       </c>
       <c r="B28" t="n">
@@ -25574,7 +25562,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" t="n">
         <v>28</v>
       </c>
       <c r="B29" t="n">
@@ -25720,7 +25708,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" t="n">
         <v>29</v>
       </c>
       <c r="B30" t="n">
@@ -25866,7 +25854,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" t="n">
         <v>30</v>
       </c>
       <c r="B31" t="n">
@@ -26012,7 +26000,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" t="n">
         <v>31</v>
       </c>
       <c r="B32" t="n">
@@ -26158,7 +26146,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" t="n">
         <v>32</v>
       </c>
       <c r="B33" t="n">
@@ -26304,7 +26292,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" t="n">
         <v>33</v>
       </c>
       <c r="B34" t="n">
@@ -26450,7 +26438,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" t="n">
         <v>34</v>
       </c>
       <c r="B35" t="n">
@@ -26596,7 +26584,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" t="n">
         <v>35</v>
       </c>
       <c r="B36" t="n">
@@ -26742,7 +26730,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" t="n">
         <v>36</v>
       </c>
       <c r="B37" t="n">
@@ -26888,7 +26876,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" t="n">
         <v>37</v>
       </c>
       <c r="B38" t="n">
@@ -27034,7 +27022,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" t="n">
         <v>38</v>
       </c>
       <c r="B39" t="n">
@@ -27180,7 +27168,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" t="n">
         <v>39</v>
       </c>
       <c r="B40" t="n">
@@ -27326,7 +27314,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" t="n">
         <v>40</v>
       </c>
       <c r="B41" t="n">
@@ -27472,7 +27460,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" t="n">
         <v>41</v>
       </c>
       <c r="B42" t="n">
@@ -27618,7 +27606,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" t="n">
         <v>42</v>
       </c>
       <c r="B43" t="n">
@@ -27764,7 +27752,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" t="n">
         <v>43</v>
       </c>
       <c r="B44" t="n">
@@ -27910,7 +27898,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" t="n">
         <v>44</v>
       </c>
       <c r="B45" t="n">
@@ -28056,7 +28044,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" t="n">
         <v>45</v>
       </c>
       <c r="B46" t="n">
@@ -28202,7 +28190,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" t="n">
         <v>46</v>
       </c>
       <c r="B47" t="n">
@@ -28348,7 +28336,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" t="n">
         <v>47</v>
       </c>
       <c r="B48" t="n">

</xml_diff>